<commit_message>
update: add Case Study sheet with graduate profile, skills matrix, and pipeline outcome
</commit_message>
<xml_diff>
--- a/UK_Graduate_Talent_Pipeline_Analysis.xlsx
+++ b/UK_Graduate_Talent_Pipeline_Analysis.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Attainment Evidence" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Scenario Model" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Findings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Case Study - Graduate Profile" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,8 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -88,7 +90,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -142,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +181,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2361,4 +2375,1168 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Case Study: Single Graduate Pipeline Journey</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>One data point in the pipeline. Update blue cells to model any graduate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>GRADUATE PROFILE (Updateable)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Pawan Singh Kapkoti</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Nationality</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Qualification</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>MSc Data Analytics</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Aston University, 2:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Graduation date</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>March 2024</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Visa type</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>PSW (Graduate Route)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>2 year duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Visa expiry</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Days remaining (as of analysis)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Auto-update when reviewing</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Certifications earned in UK</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>PL-300, Google Data Analytics</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Self-funded, self-studied</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Portfolio projects built</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="8" t="inlineStr"/>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>All public on GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Target role</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>Data Analyst / Data Engineer</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>SOC 3544 / 3133</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Target salary</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>28000</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>GBP/yr</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Entry level data analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>INVESTMENT INTO UK ECONOMY</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Amount (GBP)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Recipient</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>MSc tuition fee</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Aston University</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Student visa fee</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Home Office</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Government fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>NHS surcharge (student, 1 year)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>776</v>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>NHS / Treasury</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Healthcare access</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>PSW visa fee</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>822</v>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Home Office</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Government fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>NHS surcharge (PSW, 2 years)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>2070</v>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>NHS / Treasury</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Healthcare access</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Living costs (rent, food, bills - 30 months)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>UK landlords, businesses</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Consumer spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>PL-300 exam fee</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>165</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Microsoft (UK operation)</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Income tax paid (20 months employment)</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>HMRC</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Tax revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>National Insurance paid (20 months)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>HMRC</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Tax revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Council tax paid (20 months)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Hull City Council</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Local government</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL INVESTED INTO UK</t>
+        </is>
+      </c>
+      <c r="B31" s="28">
+        <f>SUM(B21:B30)</f>
+        <v/>
+      </c>
+      <c r="C31" s="8" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>WHAT THE UK GOT BACK</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Tax + NI contributed</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>5600</v>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Payslip data</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Consumer spending in UK economy</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Rent, food, transport, retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>NHS services consumed</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>One A&amp;E visit (estimated NHS cost)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Prescription cost paid by graduate</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Out of pocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>NHS payments made (NI share + IHS)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>4609</v>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>NI allocation + Immigration Health Surcharge</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>NHS payment-to-usage ratio</t>
+        </is>
+      </c>
+      <c r="B40" s="29">
+        <f>B39/B37</f>
+        <v/>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Net NHS surplus from this graduate</t>
+        </is>
+      </c>
+      <c r="B41" s="10">
+        <f>B39-B37</f>
+        <v/>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Total tax + fees paid to government</t>
+        </is>
+      </c>
+      <c r="B42" s="10">
+        <f>B35+B39+B21+B22+B23+B24</f>
+        <v/>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Tuition paid to university</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL UK REVENUE FROM THIS GRADUATE</t>
+        </is>
+      </c>
+      <c r="B44" s="10">
+        <f>B42+B43</f>
+        <v/>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>EMPLOYABILITY ASSESSMENT</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="n"/>
+      <c r="D46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Skill / Qualification</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Relevance</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>MSc Data Analytics (2:1)</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Aston University transcript</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Core qualification</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft PL-300 (Power BI)</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Credential ID: C2A34AA4132D8722</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Industry certification</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>Online verifiable</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Google Data Analytics Certificate</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Coursera — 8 courses</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Industry training</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Verifiable</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Python (pandas, scikit-learn, matplotlib)</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>10 GitHub projects with executed notebooks</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Primary language for data roles</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Public repos</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>SQL (window functions, CTEs, aggregations)</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>14 analytical queries on GitHub</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Required for all data roles</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Public repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>dbt (Core)</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>11 models, 94 automated tests across 2 projects</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Growing demand in data engineering</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Public repos</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>PL-300 certified + dashboard in Apex project</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Most requested BI tool in UK</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Verifiable</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>3 projects using PostgreSQL (local + Neon cloud)</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Standard database</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Public repos</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI/CD</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>3 workflows: lint, test, scheduled ingest</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>DevOps capability</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Public repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Docker</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Dockerfile in Apex project</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Containerisation</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Public repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>AWS (S3, Glue, Athena)</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Crime Analysis project on AWS</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Cloud platform</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>Public repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Excel (advanced formulas, charts)</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Employment analysis + case study workbook</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Required for analyst roles</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Public repo</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Streamlit</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Live deployed dashboard</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Data app framework</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>Live URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>ERP systems (SI Integreater)</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>12 months daily operational use</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Production environment experience</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Employer reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Team leadership</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>Managing 11+ operatives at Copernus</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Soft skill</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Employer reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>PIPELINE OUTCOME</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="4" t="n"/>
+      <c r="D64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>Skilled Worker visa salary threshold</t>
+        </is>
+      </c>
+      <c r="B65" s="22">
+        <f>'Model Inputs'!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="20" t="inlineStr">
+        <is>
+          <t>Graduate's target salary</t>
+        </is>
+      </c>
+      <c r="B66" s="30" t="n">
+        <v>28000</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>Salary gap</t>
+        </is>
+      </c>
+      <c r="B67" s="31">
+        <f>B65-B66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="inlineStr">
+        <is>
+          <t>Can this graduate qualify for Skilled Worker visa?</t>
+        </is>
+      </c>
+      <c r="B68" s="32">
+        <f>IF(B67&gt;0,"NO - Salary gap of "&amp;TEXT(B67,"#,##0")&amp;" prevents sponsorship","YES")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="33" t="inlineStr">
+        <is>
+          <t>CONCLUSION</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="20" t="inlineStr">
+        <is>
+          <t>This graduate invested 51,523 into the UK economy. They hold a postgraduate degree,</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="20" t="inlineStr">
+        <is>
+          <t>an industry certification, 15 verified technical skills, and 10 portfolio projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>The salary threshold prevents them from staying. The pipeline loses this talent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>This is one case. Multiply by 100,000 graduates per year.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>